<commit_message>
Mise a jour des README et des scripts
</commit_message>
<xml_diff>
--- a/P12_Pricer_autocall/autocall_pricer.xlsx
+++ b/P12_Pricer_autocall/autocall_pricer.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rasqu\Desktop\Quant_Project\P12 Pricer autocall\V1\files 12. Pricer de produit structuré autocall (AthenaPhoenix)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rasqu\Desktop\Quant_ProjectGit\P12_Pricer_autocall\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3F497CC9AC84F1F7F851F33B2B201E73E13A7253" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D1AC386-D550-423A-8532-73A919F94517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -159,7 +159,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +217,12 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -267,8 +273,6 @@
   </cellStyleXfs>
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -289,6 +293,8 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,6 +880,10 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -912,6 +922,81 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>523875</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>4763</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>176213</xdr:colOff>
+          <xdr:row>8</xdr:row>
+          <xdr:rowOff>95250</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2049" name="Button 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2049"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000001080000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="45720" tIns="45720" rIns="45720" bIns="45720" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="fr-FR" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri"/>
+                  <a:ea typeface="Calibri"/>
+                  <a:cs typeface="Calibri"/>
+                </a:rPr>
+                <a:t>RunPricing</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData fPrintsWithSheet="0"/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -1104,123 +1189,123 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.649999999999999" x14ac:dyDescent="0.5">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5">
-        <v>100</v>
+      <c r="C5" s="3">
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="4">
         <v>1000</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="7">
-        <v>0.03</v>
+      <c r="C7" s="5">
+        <v>0.06</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="5">
         <v>0.02</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="5">
         <v>0.22</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="6">
         <v>0.7</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="6">
         <v>0.7</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="5">
         <v>0.08</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1244,510 +1329,510 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="17.649999999999999" x14ac:dyDescent="0.5">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B5" s="13">
+      <c r="B5" s="11">
         <v>0.3</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="12">
         <f>B5*Inputs!$C$5</f>
-        <v>30</v>
-      </c>
-      <c r="D5" s="15">
+        <v>60</v>
+      </c>
+      <c r="D5" s="13">
         <f>IF(C5&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C5/Inputs!$C$5)</f>
         <v>300</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="13">
         <f>IF(C5&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="13">
         <f t="shared" ref="F5:F27" si="0">D5+E5</f>
         <v>300</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B6" s="13">
+      <c r="B6" s="11">
         <v>0.35</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="12">
         <f>B6*Inputs!$C$5</f>
-        <v>35</v>
-      </c>
-      <c r="D6" s="15">
+        <v>70</v>
+      </c>
+      <c r="D6" s="13">
         <f>IF(C6&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C6/Inputs!$C$5)</f>
         <v>350</v>
       </c>
-      <c r="E6" s="15">
+      <c r="E6" s="13">
         <f>IF(C6&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="15">
+      <c r="F6" s="13">
         <f t="shared" si="0"/>
         <v>350</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B7" s="13">
+      <c r="B7" s="11">
         <v>0.4</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="12">
         <f>B7*Inputs!$C$5</f>
-        <v>40</v>
-      </c>
-      <c r="D7" s="15">
+        <v>80</v>
+      </c>
+      <c r="D7" s="13">
         <f>IF(C7&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C7/Inputs!$C$5)</f>
         <v>400</v>
       </c>
-      <c r="E7" s="15">
+      <c r="E7" s="13">
         <f>IF(C7&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="13">
         <f t="shared" si="0"/>
         <v>400</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B8" s="13">
+      <c r="B8" s="11">
         <v>0.45</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="12">
         <f>B8*Inputs!$C$5</f>
-        <v>45</v>
-      </c>
-      <c r="D8" s="15">
+        <v>90</v>
+      </c>
+      <c r="D8" s="13">
         <f>IF(C8&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C8/Inputs!$C$5)</f>
         <v>450</v>
       </c>
-      <c r="E8" s="15">
+      <c r="E8" s="13">
         <f>IF(C8&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="13">
         <f t="shared" si="0"/>
         <v>450</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B9" s="13">
+      <c r="B9" s="11">
         <v>0.5</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="12">
         <f>B9*Inputs!$C$5</f>
-        <v>50</v>
-      </c>
-      <c r="D9" s="15">
+        <v>100</v>
+      </c>
+      <c r="D9" s="13">
         <f>IF(C9&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C9/Inputs!$C$5)</f>
         <v>500</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="13">
         <f>IF(C9&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="13">
         <f t="shared" si="0"/>
         <v>500</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B10" s="13">
+      <c r="B10" s="11">
         <v>0.55000000000000004</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="12">
         <f>B10*Inputs!$C$5</f>
-        <v>55.000000000000007</v>
-      </c>
-      <c r="D10" s="15">
+        <v>110.00000000000001</v>
+      </c>
+      <c r="D10" s="13">
         <f>IF(C10&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C10/Inputs!$C$5)</f>
         <v>550.00000000000011</v>
       </c>
-      <c r="E10" s="15">
+      <c r="E10" s="13">
         <f>IF(C10&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="13">
         <f t="shared" si="0"/>
         <v>550.00000000000011</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B11" s="13">
+      <c r="B11" s="11">
         <v>0.6</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="12">
         <f>B11*Inputs!$C$5</f>
-        <v>60</v>
-      </c>
-      <c r="D11" s="15">
+        <v>120</v>
+      </c>
+      <c r="D11" s="13">
         <f>IF(C11&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C11/Inputs!$C$5)</f>
         <v>600</v>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="13">
         <f>IF(C11&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="13">
         <f t="shared" si="0"/>
         <v>600</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B12" s="13">
+      <c r="B12" s="11">
         <v>0.65</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="12">
         <f>B12*Inputs!$C$5</f>
-        <v>65</v>
-      </c>
-      <c r="D12" s="15">
+        <v>130</v>
+      </c>
+      <c r="D12" s="13">
         <f>IF(C12&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C12/Inputs!$C$5)</f>
         <v>650</v>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="13">
         <f>IF(C12&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="13">
         <f t="shared" si="0"/>
         <v>650</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B13" s="13">
+      <c r="B13" s="11">
         <v>0.7</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="12">
         <f>B13*Inputs!$C$5</f>
-        <v>70</v>
-      </c>
-      <c r="D13" s="15">
+        <v>140</v>
+      </c>
+      <c r="D13" s="13">
         <f>IF(C13&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C13/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="13">
         <f>IF(C13&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B14" s="13">
+      <c r="B14" s="11">
         <v>0.75</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="12">
         <f>B14*Inputs!$C$5</f>
-        <v>75</v>
-      </c>
-      <c r="D14" s="15">
+        <v>150</v>
+      </c>
+      <c r="D14" s="13">
         <f>IF(C14&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C14/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E14" s="15">
+      <c r="E14" s="13">
         <f>IF(C14&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B15" s="13">
+      <c r="B15" s="11">
         <v>0.8</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="12">
         <f>B15*Inputs!$C$5</f>
-        <v>80</v>
-      </c>
-      <c r="D15" s="15">
+        <v>160</v>
+      </c>
+      <c r="D15" s="13">
         <f>IF(C15&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C15/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="13">
         <f>IF(C15&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B16" s="13">
+      <c r="B16" s="11">
         <v>0.85</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="12">
         <f>B16*Inputs!$C$5</f>
-        <v>85</v>
-      </c>
-      <c r="D16" s="15">
+        <v>170</v>
+      </c>
+      <c r="D16" s="13">
         <f>IF(C16&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C16/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="13">
         <f>IF(C16&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F16" s="15">
+      <c r="F16" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B17" s="13">
+      <c r="B17" s="11">
         <v>0.9</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="12">
         <f>B17*Inputs!$C$5</f>
-        <v>90</v>
-      </c>
-      <c r="D17" s="15">
+        <v>180</v>
+      </c>
+      <c r="D17" s="13">
         <f>IF(C17&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C17/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="13">
         <f>IF(C17&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F17" s="15">
+      <c r="F17" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B18" s="13">
+      <c r="B18" s="11">
         <v>0.95</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="12">
         <f>B18*Inputs!$C$5</f>
-        <v>95</v>
-      </c>
-      <c r="D18" s="15">
+        <v>190</v>
+      </c>
+      <c r="D18" s="13">
         <f>IF(C18&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C18/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="13">
         <f>IF(C18&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F18" s="15">
+      <c r="F18" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B19" s="13">
+      <c r="B19" s="11">
         <v>1</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="12">
         <f>B19*Inputs!$C$5</f>
-        <v>100</v>
-      </c>
-      <c r="D19" s="15">
+        <v>200</v>
+      </c>
+      <c r="D19" s="13">
         <f>IF(C19&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C19/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E19" s="15">
+      <c r="E19" s="13">
         <f>IF(C19&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F19" s="15">
+      <c r="F19" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B20" s="13">
+      <c r="B20" s="11">
         <v>1.05</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="12">
         <f>B20*Inputs!$C$5</f>
-        <v>105</v>
-      </c>
-      <c r="D20" s="15">
+        <v>210</v>
+      </c>
+      <c r="D20" s="13">
         <f>IF(C20&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C20/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="13">
         <f>IF(C20&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B21" s="13">
+      <c r="B21" s="11">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="12">
         <f>B21*Inputs!$C$5</f>
-        <v>110.00000000000001</v>
-      </c>
-      <c r="D21" s="15">
+        <v>220.00000000000003</v>
+      </c>
+      <c r="D21" s="13">
         <f>IF(C21&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C21/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="13">
         <f>IF(C21&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B22" s="13">
+      <c r="B22" s="11">
         <v>1.1499999999999999</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="12">
         <f>B22*Inputs!$C$5</f>
-        <v>114.99999999999999</v>
-      </c>
-      <c r="D22" s="15">
+        <v>229.99999999999997</v>
+      </c>
+      <c r="D22" s="13">
         <f>IF(C22&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C22/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="13">
         <f>IF(C22&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F22" s="15">
+      <c r="F22" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B23" s="13">
+      <c r="B23" s="11">
         <v>1.2</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="12">
         <f>B23*Inputs!$C$5</f>
-        <v>120</v>
-      </c>
-      <c r="D23" s="15">
+        <v>240</v>
+      </c>
+      <c r="D23" s="13">
         <f>IF(C23&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C23/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="13">
         <f>IF(C23&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B24" s="13">
+      <c r="B24" s="11">
         <v>1.25</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="12">
         <f>B24*Inputs!$C$5</f>
-        <v>125</v>
-      </c>
-      <c r="D24" s="15">
+        <v>250</v>
+      </c>
+      <c r="D24" s="13">
         <f>IF(C24&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C24/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="13">
         <f>IF(C24&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B25" s="13">
+      <c r="B25" s="11">
         <v>1.3</v>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="12">
         <f>B25*Inputs!$C$5</f>
-        <v>130</v>
-      </c>
-      <c r="D25" s="15">
+        <v>260</v>
+      </c>
+      <c r="D25" s="13">
         <f>IF(C25&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C25/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="13">
         <f>IF(C25&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B26" s="13">
+      <c r="B26" s="11">
         <v>1.35</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="12">
         <f>B26*Inputs!$C$5</f>
-        <v>135</v>
-      </c>
-      <c r="D26" s="15">
+        <v>270</v>
+      </c>
+      <c r="D26" s="13">
         <f>IF(C26&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C26/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="13">
         <f>IF(C26&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B27" s="13">
+      <c r="B27" s="11">
         <v>1.4</v>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="12">
         <f>B27*Inputs!$C$5</f>
-        <v>140</v>
-      </c>
-      <c r="D27" s="15">
+        <v>280</v>
+      </c>
+      <c r="D27" s="13">
         <f>IF(C27&gt;=Inputs!$C$12*Inputs!$C$5,Inputs!$C$6,Inputs!$C$6*C27/Inputs!$C$5)</f>
         <v>1000</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="13">
         <f>IF(C27&gt;=Inputs!$C$11*Inputs!$C$5,Inputs!$C$13*Inputs!$C$6,0)</f>
         <v>80</v>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="13">
         <f t="shared" si="0"/>
         <v>1080</v>
       </c>
@@ -1763,7 +1848,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Feuil3"/>
   <dimension ref="B2:F18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1774,111 +1859,111 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" ht="17.649999999999999" x14ac:dyDescent="0.5">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
     </row>
     <row r="4" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="17">
-        <v>1000.12</v>
+      <c r="C7" s="15">
+        <v>972.77511946462562</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B8" s="16" t="s">
+      <c r="B8" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="18">
-        <v>1.0001</v>
+      <c r="C8" s="16">
+        <v>0.97277511946462558</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="19">
-        <v>0.34</v>
+      <c r="C9" s="17">
+        <v>1.0800289688932467</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="18">
         <v>2.9975000000000001</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="19">
         <v>0.59299999999999997</v>
       </c>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="19">
         <v>0.17100000000000001</v>
       </c>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="17">
         <v>1.93</v>
       </c>
     </row>
     <row r="15" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="16" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="22">
+      <c r="C16" s="20">
         <v>0.47399999999999998</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="20">
         <v>0.11899999999999999</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.45">
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="22">
+      <c r="C18" s="20">
         <v>0.40699999999999997</v>
       </c>
     </row>
@@ -1888,6 +1973,36 @@
     <mergeCell ref="B4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="2049" r:id="rId4" name="Button 1">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!RunPricing">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>4</xdr:col>
+                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:row>5</xdr:row>
+                    <xdr:rowOff>4763</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>7</xdr:col>
+                    <xdr:colOff>176213</xdr:colOff>
+                    <xdr:row>8</xdr:row>
+                    <xdr:rowOff>95250</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
 </worksheet>
 </file>
</xml_diff>